<commit_message>
XlsxExporter shows "Data collected" and "Report generated" cells
</commit_message>
<xml_diff>
--- a/tests/anki_addons_dataset/exporter/xlsx/exp_aggregation.xlsx
+++ b/tests/anki_addons_dataset/exporter/xlsx/exp_aggregation.xlsx
@@ -20,9 +20,21 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t xml:space="preserve">Anki Addons Dataset</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data collected:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-10-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Report generated:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025-01-25</t>
   </si>
   <si>
     <t xml:space="preserve">Property</t>
@@ -47,10 +59,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -80,6 +93,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b val="true"/>
@@ -135,16 +154,36 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -341,62 +380,83 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="40.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20.71"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="22.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3"/>
+      <c r="E1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="4"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="I1" s="3"/>
+      <c r="J1" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="K1" s="6"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="2" t="s">
+      <c r="A3" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="1" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="0" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="0" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" s="0" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7" s="0" t="n">
-        <v>2</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="5">
     <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="J1:K1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>